<commit_message>
fix: close phase 00 round 3 review findings
</commit_message>
<xml_diff>
--- a/tests/fixtures/locations.xlsx
+++ b/tests/fixtures/locations.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Limits" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Limits" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -18,10 +19,35 @@
   <si>
     <t>travel</t>
   </si>
+  <si>
+    <r>
+      <t>Summary &amp;</t>
+    </r>
+    <r>
+      <t> policy</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2">
+        <v>999</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">

</xml_diff>